<commit_message>
Made some Squares Grid Winners 2024
</commit_message>
<xml_diff>
--- a/scripts/SquareGridWinners_2024.xlsx
+++ b/scripts/SquareGridWinners_2024.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\fundraising\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC36DD3B-5A1E-47D1-9D21-67AE1FB66A12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E9A6DF8-28AE-4B82-ACC4-63979FD5318A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{088BB7A9-5091-48E0-BF05-ED8B2D8B8665}"/>
+    <workbookView xWindow="3228" yWindow="264" windowWidth="15636" windowHeight="10884" activeTab="1" xr2:uid="{088BB7A9-5091-48E0-BF05-ED8B2D8B8665}"/>
   </bookViews>
   <sheets>
     <sheet name="PCDWBA_6_1" sheetId="2" r:id="rId1"/>
@@ -4776,20 +4776,32 @@
       <c r="F62" s="1">
         <v>1</v>
       </c>
+      <c r="G62" s="1">
+        <v>222</v>
+      </c>
+      <c r="H62" s="1">
+        <v>191</v>
+      </c>
       <c r="I62" s="1">
         <f>MOD(K62,10)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J62" s="1">
         <f>MOD(L62,10)</f>
         <v>0</v>
       </c>
+      <c r="K62" s="1">
+        <v>63</v>
+      </c>
+      <c r="L62" s="1">
+        <v>50</v>
+      </c>
       <c r="M62" s="1" t="s">
         <v>12</v>
       </c>
       <c r="O62" t="str">
         <f t="shared" si="3"/>
-        <v>insert into squaregridwinners values ('PCDWBA',2024,6,1,5,1,,,0,0,,,'Y');</v>
+        <v>insert into squaregridwinners values ('PCDWBA',2024,6,1,5,1,222,191,3,0,63,50,'Y');</v>
       </c>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.3">
@@ -4811,20 +4823,32 @@
       <c r="F63" s="1">
         <v>2</v>
       </c>
+      <c r="G63" s="1">
+        <v>58</v>
+      </c>
+      <c r="H63" s="1">
+        <v>3</v>
+      </c>
       <c r="I63" s="1">
         <f t="shared" ref="I63" si="6">MOD(K63,10)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J63" s="1">
         <f t="shared" ref="J63" si="7">MOD(L63,10)</f>
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="K63" s="1">
+        <v>86</v>
+      </c>
+      <c r="L63" s="1">
+        <v>72</v>
       </c>
       <c r="M63" s="1" t="s">
         <v>12</v>
       </c>
       <c r="O63" t="str">
         <f t="shared" si="3"/>
-        <v>insert into squaregridwinners values ('PCDWBA',2024,6,1,5,2,,,0,0,,,'Y');</v>
+        <v>insert into squaregridwinners values ('PCDWBA',2024,6,1,5,2,58,3,6,2,86,72,'Y');</v>
       </c>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.3">
@@ -7769,20 +7793,32 @@
       <c r="F62" s="1">
         <v>1</v>
       </c>
+      <c r="G62" s="1">
+        <v>250</v>
+      </c>
+      <c r="H62" s="1">
+        <v>191</v>
+      </c>
       <c r="I62" s="1">
         <f t="shared" ref="I62:I63" si="7">MOD(K62,10)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J62" s="1">
         <f t="shared" ref="J62:J63" si="8">MOD(L62,10)</f>
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="K62" s="1">
+        <v>78</v>
+      </c>
+      <c r="L62" s="1">
+        <v>59</v>
       </c>
       <c r="M62" s="1" t="s">
         <v>12</v>
       </c>
       <c r="O62" t="str">
         <f t="shared" ref="O62:O63" si="9">CONCATENATE("insert into squaregridwinners values ('",A62,"',",B62,",",C62,",",D62,",",E62,",",F62,",",G62,",",H62,",",I62,",",J62,",",K62,",",L62,",'",M62,"');")</f>
-        <v>insert into squaregridwinners values ('PCDWBA',2024,7,2,5,1,,,0,0,,,'Y');</v>
+        <v>insert into squaregridwinners values ('PCDWBA',2024,7,2,5,1,250,191,8,9,78,59,'Y');</v>
       </c>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.3">
@@ -7804,20 +7840,32 @@
       <c r="F63" s="1">
         <v>2</v>
       </c>
+      <c r="G63" s="1">
+        <v>120</v>
+      </c>
+      <c r="H63" s="1">
+        <v>58</v>
+      </c>
       <c r="I63" s="1">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J63" s="1">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="K63" s="1">
+        <v>71</v>
+      </c>
+      <c r="L63" s="1">
+        <v>69</v>
       </c>
       <c r="M63" s="1" t="s">
         <v>12</v>
       </c>
       <c r="O63" t="str">
         <f t="shared" si="9"/>
-        <v>insert into squaregridwinners values ('PCDWBA',2024,7,2,5,2,,,0,0,,,'Y');</v>
+        <v>insert into squaregridwinners values ('PCDWBA',2024,7,2,5,2,120,58,1,9,71,69,'Y');</v>
       </c>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.3">
@@ -10666,20 +10714,32 @@
       <c r="F62" s="1">
         <v>1</v>
       </c>
-      <c r="I62" s="1">
-        <f t="shared" ref="I62:I63" si="5">MOD(K62,10)</f>
+      <c r="G62" s="2">
+        <v>222</v>
+      </c>
+      <c r="H62" s="2">
+        <v>191</v>
+      </c>
+      <c r="I62" s="2">
+        <f>MOD(K62,10)</f>
+        <v>3</v>
+      </c>
+      <c r="J62" s="2">
+        <f>MOD(L62,10)</f>
         <v>0</v>
       </c>
-      <c r="J62" s="1">
-        <f t="shared" ref="J62:J63" si="6">MOD(L62,10)</f>
-        <v>0</v>
+      <c r="K62" s="2">
+        <v>63</v>
+      </c>
+      <c r="L62" s="2">
+        <v>50</v>
       </c>
       <c r="M62" s="1" t="s">
         <v>12</v>
       </c>
       <c r="O62" t="str">
-        <f t="shared" ref="O62:O63" si="7">CONCATENATE("insert into squaregridwinners values ('",A62,"',",B62,",",C62,",",D62,",",E62,",",F62,",",G62,",",H62,",",I62,",",J62,",",K62,",",L62,",'",M62,"');")</f>
-        <v>insert into squaregridwinners values ('SCDDGC',2024,6,1,5,1,,,0,0,,,'Y');</v>
+        <f t="shared" ref="O62:O63" si="5">CONCATENATE("insert into squaregridwinners values ('",A62,"',",B62,",",C62,",",D62,",",E62,",",F62,",",G62,",",H62,",",I62,",",J62,",",K62,",",L62,",'",M62,"');")</f>
+        <v>insert into squaregridwinners values ('SCDDGC',2024,6,1,5,1,222,191,3,0,63,50,'Y');</v>
       </c>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.3">
@@ -10701,20 +10761,32 @@
       <c r="F63" s="1">
         <v>2</v>
       </c>
-      <c r="I63" s="1">
+      <c r="G63" s="3">
+        <v>58</v>
+      </c>
+      <c r="H63" s="3">
+        <v>3</v>
+      </c>
+      <c r="I63" s="3">
+        <f t="shared" ref="I63:J63" si="6">MOD(K63,10)</f>
+        <v>6</v>
+      </c>
+      <c r="J63" s="3">
+        <f t="shared" si="6"/>
+        <v>2</v>
+      </c>
+      <c r="K63" s="3">
+        <v>86</v>
+      </c>
+      <c r="L63" s="3">
+        <v>72</v>
+      </c>
+      <c r="M63" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O63" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J63" s="1">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="M63" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="O63" t="str">
-        <f t="shared" si="7"/>
-        <v>insert into squaregridwinners values ('SCDDGC',2024,6,1,5,2,,,0,0,,,'Y');</v>
+        <v>insert into squaregridwinners values ('SCDDGC',2024,6,1,5,2,58,3,6,2,86,72,'Y');</v>
       </c>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.3">
@@ -10737,18 +10809,18 @@
         <v>1</v>
       </c>
       <c r="I64" s="1">
-        <f t="shared" ref="I64" si="8">MOD(K64,10)</f>
+        <f t="shared" ref="I64" si="7">MOD(K64,10)</f>
         <v>0</v>
       </c>
       <c r="J64" s="1">
-        <f t="shared" ref="J64" si="9">MOD(L64,10)</f>
+        <f t="shared" ref="J64" si="8">MOD(L64,10)</f>
         <v>0</v>
       </c>
       <c r="M64" s="1" t="s">
         <v>12</v>
       </c>
       <c r="O64" t="str">
-        <f t="shared" ref="O64" si="10">CONCATENATE("insert into squaregridwinners values ('",A64,"',",B64,",",C64,",",D64,",",E64,",",F64,",",G64,",",H64,",",I64,",",J64,",",K64,",",L64,",'",M64,"');")</f>
+        <f t="shared" ref="O64" si="9">CONCATENATE("insert into squaregridwinners values ('",A64,"',",B64,",",C64,",",D64,",",E64,",",F64,",",G64,",",H64,",",I64,",",J64,",",K64,",",L64,",'",M64,"');")</f>
         <v>insert into squaregridwinners values ('SCDDGC',2024,6,1,6,1,,,0,0,,,'Y');</v>
       </c>
     </row>
@@ -13563,20 +13635,32 @@
       <c r="F62" s="1">
         <v>1</v>
       </c>
-      <c r="I62" s="1">
+      <c r="G62" s="2">
+        <v>222</v>
+      </c>
+      <c r="H62" s="2">
+        <v>191</v>
+      </c>
+      <c r="I62" s="2">
         <f>MOD(K62,10)</f>
-        <v>0</v>
-      </c>
-      <c r="J62" s="1">
+        <v>3</v>
+      </c>
+      <c r="J62" s="2">
         <f>MOD(L62,10)</f>
         <v>0</v>
       </c>
+      <c r="K62" s="2">
+        <v>63</v>
+      </c>
+      <c r="L62" s="2">
+        <v>50</v>
+      </c>
       <c r="M62" s="1" t="s">
         <v>12</v>
       </c>
       <c r="O62" t="str">
         <f t="shared" ref="O62:O63" si="5">CONCATENATE("insert into squaregridwinners values ('",A62,"',",B62,",",C62,",",D62,",",E62,",",F62,",",G62,",",H62,",",I62,",",J62,",",K62,",",L62,",'",M62,"');")</f>
-        <v>insert into squaregridwinners values ('USADVB',2024,6,2,5,1,,,0,0,,,'Y');</v>
+        <v>insert into squaregridwinners values ('USADVB',2024,6,2,5,1,222,191,3,0,63,50,'Y');</v>
       </c>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.3">
@@ -13598,20 +13682,32 @@
       <c r="F63" s="1">
         <v>2</v>
       </c>
-      <c r="I63" s="1">
-        <f t="shared" ref="I63" si="6">MOD(K63,10)</f>
-        <v>0</v>
-      </c>
-      <c r="J63" s="1">
-        <f t="shared" ref="J63" si="7">MOD(L63,10)</f>
-        <v>0</v>
+      <c r="G63" s="3">
+        <v>58</v>
+      </c>
+      <c r="H63" s="3">
+        <v>3</v>
+      </c>
+      <c r="I63" s="3">
+        <f t="shared" ref="I63:J63" si="6">MOD(K63,10)</f>
+        <v>6</v>
+      </c>
+      <c r="J63" s="3">
+        <f t="shared" si="6"/>
+        <v>2</v>
+      </c>
+      <c r="K63" s="3">
+        <v>86</v>
+      </c>
+      <c r="L63" s="3">
+        <v>72</v>
       </c>
       <c r="M63" s="1" t="s">
         <v>12</v>
       </c>
       <c r="O63" t="str">
         <f t="shared" si="5"/>
-        <v>insert into squaregridwinners values ('USADVB',2024,6,2,5,2,,,0,0,,,'Y');</v>
+        <v>insert into squaregridwinners values ('USADVB',2024,6,2,5,2,58,3,6,2,86,72,'Y');</v>
       </c>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.3">
@@ -13645,7 +13741,7 @@
         <v>12</v>
       </c>
       <c r="O64" t="str">
-        <f t="shared" ref="O64" si="8">CONCATENATE("insert into squaregridwinners values ('",A64,"',",B64,",",C64,",",D64,",",E64,",",F64,",",G64,",",H64,",",I64,",",J64,",",K64,",",L64,",'",M64,"');")</f>
+        <f t="shared" ref="O64" si="7">CONCATENATE("insert into squaregridwinners values ('",A64,"',",B64,",",C64,",",D64,",",E64,",",F64,",",G64,",",H64,",",I64,",",J64,",",K64,",",L64,",'",M64,"');")</f>
         <v>insert into squaregridwinners values ('USADVB',2024,6,2,6,1,,,0,0,,,'Y');</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add new message to notify users if no event occurs
</commit_message>
<xml_diff>
--- a/scripts/SquareGridWinners_2024.xlsx
+++ b/scripts/SquareGridWinners_2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\fundraising\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E9A6DF8-28AE-4B82-ACC4-63979FD5318A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D60DB17F-ABE8-4145-A3A7-A7A0A5B6F7F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3228" yWindow="264" windowWidth="15636" windowHeight="10884" activeTab="1" xr2:uid="{088BB7A9-5091-48E0-BF05-ED8B2D8B8665}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{088BB7A9-5091-48E0-BF05-ED8B2D8B8665}"/>
   </bookViews>
   <sheets>
     <sheet name="PCDWBA_6_1" sheetId="2" r:id="rId1"/>
@@ -4870,20 +4870,32 @@
       <c r="F64" s="1">
         <v>1</v>
       </c>
+      <c r="G64" s="1">
+        <v>58</v>
+      </c>
+      <c r="H64" s="1">
+        <v>222</v>
+      </c>
       <c r="I64" s="1">
         <f>MOD(K64,10)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J64" s="1">
         <f>MOD(L64,10)</f>
         <v>0</v>
       </c>
+      <c r="K64" s="1">
+        <v>75</v>
+      </c>
+      <c r="L64" s="1">
+        <v>60</v>
+      </c>
       <c r="M64" s="1" t="s">
         <v>12</v>
       </c>
       <c r="O64" t="str">
         <f t="shared" ref="O64" si="8">CONCATENATE("insert into squaregridwinners values ('",A64,"',",B64,",",C64,",",D64,",",E64,",",F64,",",G64,",",H64,",",I64,",",J64,",",K64,",",L64,",'",M64,"');")</f>
-        <v>insert into squaregridwinners values ('PCDWBA',2024,6,1,6,1,,,0,0,,,'Y');</v>
+        <v>insert into squaregridwinners values ('PCDWBA',2024,6,1,6,1,58,222,5,0,75,60,'Y');</v>
       </c>
     </row>
   </sheetData>
@@ -7887,20 +7899,32 @@
       <c r="F64" s="1">
         <v>1</v>
       </c>
+      <c r="G64" s="1">
+        <v>250</v>
+      </c>
+      <c r="H64" s="1">
+        <v>120</v>
+      </c>
       <c r="I64" s="1">
         <f t="shared" ref="I64" si="10">MOD(K64,10)</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J64" s="1">
         <f t="shared" ref="J64" si="11">MOD(L64,10)</f>
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="K64" s="1">
+        <v>87</v>
+      </c>
+      <c r="L64" s="1">
+        <v>75</v>
       </c>
       <c r="M64" s="1" t="s">
         <v>12</v>
       </c>
       <c r="O64" t="str">
         <f t="shared" ref="O64" si="12">CONCATENATE("insert into squaregridwinners values ('",A64,"',",B64,",",C64,",",D64,",",E64,",",F64,",",G64,",",H64,",",I64,",",J64,",",K64,",",L64,",'",M64,"');")</f>
-        <v>insert into squaregridwinners values ('PCDWBA',2024,7,2,6,1,,,0,0,,,'Y');</v>
+        <v>insert into squaregridwinners values ('PCDWBA',2024,7,2,6,1,250,120,7,5,87,75,'Y');</v>
       </c>
     </row>
   </sheetData>
@@ -10808,20 +10832,32 @@
       <c r="F64" s="1">
         <v>1</v>
       </c>
+      <c r="G64" s="1">
+        <v>58</v>
+      </c>
+      <c r="H64" s="1">
+        <v>222</v>
+      </c>
       <c r="I64" s="1">
-        <f t="shared" ref="I64" si="7">MOD(K64,10)</f>
+        <f>MOD(K64,10)</f>
+        <v>5</v>
+      </c>
+      <c r="J64" s="1">
+        <f>MOD(L64,10)</f>
         <v>0</v>
       </c>
-      <c r="J64" s="1">
-        <f t="shared" ref="J64" si="8">MOD(L64,10)</f>
-        <v>0</v>
+      <c r="K64" s="1">
+        <v>75</v>
+      </c>
+      <c r="L64" s="1">
+        <v>60</v>
       </c>
       <c r="M64" s="1" t="s">
         <v>12</v>
       </c>
       <c r="O64" t="str">
-        <f t="shared" ref="O64" si="9">CONCATENATE("insert into squaregridwinners values ('",A64,"',",B64,",",C64,",",D64,",",E64,",",F64,",",G64,",",H64,",",I64,",",J64,",",K64,",",L64,",'",M64,"');")</f>
-        <v>insert into squaregridwinners values ('SCDDGC',2024,6,1,6,1,,,0,0,,,'Y');</v>
+        <f t="shared" ref="O64" si="7">CONCATENATE("insert into squaregridwinners values ('",A64,"',",B64,",",C64,",",D64,",",E64,",",F64,",",G64,",",H64,",",I64,",",J64,",",K64,",",L64,",'",M64,"');")</f>
+        <v>insert into squaregridwinners values ('SCDDGC',2024,6,1,6,1,58,222,5,0,75,60,'Y');</v>
       </c>
     </row>
   </sheetData>
@@ -13729,20 +13765,32 @@
       <c r="F64" s="1">
         <v>1</v>
       </c>
+      <c r="G64" s="1">
+        <v>58</v>
+      </c>
+      <c r="H64" s="1">
+        <v>222</v>
+      </c>
       <c r="I64" s="1">
         <f>MOD(K64,10)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J64" s="1">
         <f>MOD(L64,10)</f>
         <v>0</v>
       </c>
+      <c r="K64" s="1">
+        <v>75</v>
+      </c>
+      <c r="L64" s="1">
+        <v>60</v>
+      </c>
       <c r="M64" s="1" t="s">
         <v>12</v>
       </c>
       <c r="O64" t="str">
         <f t="shared" ref="O64" si="7">CONCATENATE("insert into squaregridwinners values ('",A64,"',",B64,",",C64,",",D64,",",E64,",",F64,",",G64,",",H64,",",I64,",",J64,",",K64,",",L64,",'",M64,"');")</f>
-        <v>insert into squaregridwinners values ('USADVB',2024,6,2,6,1,,,0,0,,,'Y');</v>
+        <v>insert into squaregridwinners values ('USADVB',2024,6,2,6,1,58,222,5,0,75,60,'Y');</v>
       </c>
     </row>
   </sheetData>

</xml_diff>